<commit_message>
Calculated Average Marks for Each Subject and styled the sheet
</commit_message>
<xml_diff>
--- a/MarkSheet.xlsx
+++ b/MarkSheet.xlsx
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,31 +418,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>math</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>science</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>english</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>gym</t>
         </is>
@@ -536,6 +541,24 @@
       </c>
       <c r="E6" t="n">
         <v>60</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7">
+        <f>SUM(B2:B6)/5</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>SUM(C2:C6)/5</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>SUM(D2:D6)/5</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>SUM(E2:E6)/5</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>